<commit_message>
Added knowledge base datasets and latest chatbot updates
</commit_message>
<xml_diff>
--- a/data/official_data/knowledge/admissions.xlsx
+++ b/data/official_data/knowledge/admissions.xlsx
@@ -16,17 +16,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="140">
   <si>
     <t>Topic</t>
   </si>
   <si>
-    <t>Field</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
     <t>Source</t>
   </si>
   <si>
@@ -36,15 +30,6 @@
     <t>URL</t>
   </si>
   <si>
-    <t>General Admission</t>
-  </si>
-  <si>
-    <t>Overview</t>
-  </si>
-  <si>
-    <t>Cluster University Srinagar offers admission to various Undergraduate, Postgraduate and professional programmes through the admission process notified on its official website.</t>
-  </si>
-  <si>
     <t>Official CUS Website</t>
   </si>
   <si>
@@ -54,26 +39,434 @@
     <t>https://www.cusrinagar.edu.in</t>
   </si>
   <si>
-    <t>Official Website</t>
-  </si>
-  <si>
     <t>Admission Process</t>
   </si>
   <si>
-    <t>Admissions are conducted according to the admission notifications issued by the university. Candidates should check eligibility, submit the online application, upload required documents and complete the fee payment before the deadline.</t>
-  </si>
-  <si>
-    <t>Documents</t>
-  </si>
-  <si>
-    <t>Recent passport-size photograph, educational certificates/marksheets, domicile/category certificates (if applicable), and other documents mentioned in the admission notification.</t>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Applicable To</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Required Documents</t>
+  </si>
+  <si>
+    <t>Eligibility Basis</t>
+  </si>
+  <si>
+    <t>Admission Mode</t>
+  </si>
+  <si>
+    <t>Selection Basis</t>
+  </si>
+  <si>
+    <t>Reservation</t>
+  </si>
+  <si>
+    <t>Application Fee</t>
+  </si>
+  <si>
+    <t>Admission Portal</t>
+  </si>
+  <si>
+    <t>Important Notes</t>
+  </si>
+  <si>
+    <t>Undergraduate Admission</t>
+  </si>
+  <si>
+    <t>FYUG Admission</t>
+  </si>
+  <si>
+    <t>All Undergraduate Programmes</t>
+  </si>
+  <si>
+    <t>Admission to FYUG programmes is conducted through the Cluster University Srinagar admission portal based on CUET (UG) scores and the University's admission policy.</t>
+  </si>
+  <si>
+    <t>10th Certificate, 12th Marks Card, CUET (UG) Score Card, Aadhaar/ID Proof, Category Certificate (if applicable), Character Certificate, Migration/Transfer Certificate (if applicable), Passport-size Photograph.</t>
+  </si>
+  <si>
+    <t>10+2 or equivalent from a recognized board.</t>
+  </si>
+  <si>
+    <t>Online</t>
+  </si>
+  <si>
+    <t>CUET (UG) Merit</t>
+  </si>
+  <si>
+    <t>As per J&amp;K Government/University norms</t>
+  </si>
+  <si>
+    <t>CUS Admission Portal</t>
+  </si>
+  <si>
+    <t>Admission is provisional and subject to document verification and fulfillment of eligibility.</t>
+  </si>
+  <si>
+    <t>https://cuet.nta.nic.in ,   https://www.cusrinagar.edu.in/</t>
+  </si>
+  <si>
+    <t>Postgraduate Admission</t>
+  </si>
+  <si>
+    <t>PG Admission</t>
+  </si>
+  <si>
+    <t>All PG Programmes</t>
+  </si>
+  <si>
+    <t>Admission to postgraduate programmes is conducted through the Cluster University Srinagar admission portal. Depending on the programme, selection is based on CUET (PG) merit or merit in the qualifying examination as notified by the University.</t>
+  </si>
+  <si>
+    <t>Graduation Marks Cards, Degree/Provisional Certificate, 10th &amp; 12th Certificates, CUET (PG) Score Card (where applicable), Category Certificate, Character Certificate, Migration Certificate, Passport-size Photograph.</t>
+  </si>
+  <si>
+    <t>Bachelor's degree in the relevant discipline.</t>
+  </si>
+  <si>
+    <t>CUET (PG) Merit / Qualifying Degree Merit (programme-wise)</t>
+  </si>
+  <si>
+    <t>Rs. 700/- for the first programme and an additional Rs. 300/- for each subsequent programme.</t>
+  </si>
+  <si>
+    <t>Rs. 500/- (non-refundable) for general UG admissions, or Rs. 200/- depending on specific registration notifications.</t>
+  </si>
+  <si>
+    <t>Admission remains provisional until verification of original documents. Candidates do not need to submit physical copies of the application form or fee receipt to the university.</t>
+  </si>
+  <si>
+    <t>Integrated Programmes</t>
+  </si>
+  <si>
+    <t>IntegratedAdmission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Official CUS Website
+</t>
+  </si>
+  <si>
+    <t>Reservation Policy</t>
+  </si>
+  <si>
+    <t>All Programmes</t>
+  </si>
+  <si>
+    <t>Reservation of seats is applicable as per the latest Government of Jammu &amp; Kashmir and University reservation policy. Valid category certificates must be produced wherever applicable.</t>
+  </si>
+  <si>
+    <t>Document Verification</t>
+  </si>
+  <si>
+    <t>Admission is confirmed only after successful verification of original academic and category certificates. Any discrepancy may lead to cancellation of admission.</t>
+  </si>
+  <si>
+    <t>Fee Payment</t>
+  </si>
+  <si>
+    <t>Selected candidates must pay the prescribed admission fee online or through the mode notified by the University within the stipulated time to confirm admission.</t>
+  </si>
+  <si>
+    <t>Admissions are processed through the official Cluster University Srinagar admission portal.</t>
+  </si>
+  <si>
+    <t>Students may contact the University or the concerned constituent college for admission-related queries.</t>
+  </si>
+  <si>
+    <t>All Integrated Programmes</t>
+  </si>
+  <si>
+    <t>Admission to Integrated Programmes is conducted through the Cluster University Srinagar admission portal based on CUET (UG) merit and the University's admission policy.</t>
+  </si>
+  <si>
+    <t>10+2 or equivalent from a recognized Board with programme-specific eligibility requirements.</t>
+  </si>
+  <si>
+    <t>As per J&amp;K Government / University norms</t>
+  </si>
+  <si>
+    <t>Same as applicable programme.</t>
+  </si>
+  <si>
+    <t>Cluster University Srinagar Admission Portal</t>
+  </si>
+  <si>
+    <t>Category certificates are verified during admission. Invalid certificates may lead to cancellation of reserved category benefits.</t>
+  </si>
+  <si>
+    <t>As per latest admission notification</t>
+  </si>
+  <si>
+    <t>Admission Policy</t>
+  </si>
+  <si>
+    <t>Valid Category Certificate (if applicable).</t>
+  </si>
+  <si>
+    <t>Applicable to eligible reserved category candidates.</t>
+  </si>
+  <si>
+    <t>Merit within the applicable reservation category.</t>
+  </si>
+  <si>
+    <t>As per J&amp;K Government / University norms.</t>
+  </si>
+  <si>
+    <t>Official CUS Admission Policy</t>
+  </si>
+  <si>
+    <t>Original academic certificates, identity proof, category certificate (if applicable), migration certificate (if applicable), photographs.</t>
+  </si>
+  <si>
+    <t>Successful verification of original documents.</t>
+  </si>
+  <si>
+    <t>Offline/Online as notified.</t>
+  </si>
+  <si>
+    <t>Not Applicable</t>
+  </si>
+  <si>
+    <t>Applicable where relevant.</t>
+  </si>
+  <si>
+    <t>Admission may be cancelled if any document is found false or incorrect.</t>
+  </si>
+  <si>
+    <t>Fee payment receipt.</t>
+  </si>
+  <si>
+    <t>Selection in the admission process.</t>
+  </si>
+  <si>
+    <t>Programme-specific</t>
+  </si>
+  <si>
+    <t>Failure to pay the fee within the notified period may result in cancellation of admission.</t>
+  </si>
+  <si>
+    <t>Admission Information</t>
+  </si>
+  <si>
+    <t>Programme-specific.</t>
+  </si>
+  <si>
+    <t>As per University norms.</t>
+  </si>
+  <si>
+    <t>Applicants should regularly check the portal for notifications, merit lists and counselling updates.</t>
+  </si>
+  <si>
+    <t>Student Support</t>
+  </si>
+  <si>
+    <t>Admission Help Desk</t>
+  </si>
+  <si>
+    <t>All Applicants</t>
+  </si>
+  <si>
+    <t>Query-specific documents, if required.</t>
+  </si>
+  <si>
+    <t>Online / Offline</t>
+  </si>
+  <si>
+    <t>Applicants should use official contact details available on the University website.</t>
+  </si>
+  <si>
+    <t>Admission Cancellation</t>
+  </si>
+  <si>
+    <t>Admission may be cancelled upon withdrawal by the candidate or non-compliance with University rules.</t>
+  </si>
+  <si>
+    <t>Admission cancellation request and supporting documents, if applicable.</t>
+  </si>
+  <si>
+    <t>Refunds, if any, are governed by the University's prevailing rules.</t>
+  </si>
+  <si>
+    <t>Official University Admission Rules</t>
+  </si>
+  <si>
+    <t>Admission Documents</t>
+  </si>
+  <si>
+    <t>Migration Certificate</t>
+  </si>
+  <si>
+    <t>Students from other Universities/Boards</t>
+  </si>
+  <si>
+    <t>A migration certificate is required from candidates who have completed their qualifying examination from another University or Board, wherever applicable.</t>
+  </si>
+  <si>
+    <t>Original Migration Certificate.</t>
+  </si>
+  <si>
+    <t>Applicable where required.</t>
+  </si>
+  <si>
+    <t>Offline/Online submission</t>
+  </si>
+  <si>
+    <t>Submission timelines shall be as notified by the University.</t>
+  </si>
+  <si>
+    <t>Official Admission Notification</t>
+  </si>
+  <si>
+    <t>Student Compliance</t>
+  </si>
+  <si>
+    <t>Anti-Ragging</t>
+  </si>
+  <si>
+    <t>All Students</t>
+  </si>
+  <si>
+    <t>Submission of Anti-Ragging undertaking is mandatory as per UGC regulations.</t>
+  </si>
+  <si>
+    <t>Anti-Ragging Undertaking (Student &amp; Parent, if applicable).</t>
+  </si>
+  <si>
+    <t>Mandatory for admission confirmation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Anti-Ragging Portal</t>
+  </si>
+  <si>
+    <t>Admission may remain provisional until the undertaking is submitted.</t>
+  </si>
+  <si>
+    <t>UGC &amp; Official University Guidelines</t>
+  </si>
+  <si>
+    <t>https://www.antiragging.in/</t>
+  </si>
+  <si>
+    <t>Merit List &amp; Waiting List</t>
+  </si>
+  <si>
+    <t>Merit lists and waiting lists are published on the official University website and admission portal.</t>
+  </si>
+  <si>
+    <t>Programme-specific merit.</t>
+  </si>
+  <si>
+    <t>Merit-based.</t>
+  </si>
+  <si>
+    <t>Applicable as per norms.</t>
+  </si>
+  <si>
+    <t>Candidates must complete admission within the prescribed schedule after selection.</t>
+  </si>
+  <si>
+    <t>Official Admission Notifications</t>
+  </si>
+  <si>
+    <t>Spot Admission</t>
+  </si>
+  <si>
+    <t>Vacant Seats (if notified)</t>
+  </si>
+  <si>
+    <t>Spot admissions may be conducted by the University for vacant seats after completion of the regular admission process, subject to availability and official notification.</t>
+  </si>
+  <si>
+    <t>Same as regular admission.</t>
+  </si>
+  <si>
+    <t>Programme-specific eligibility.</t>
+  </si>
+  <si>
+    <t>Online / Offline as notified.</t>
+  </si>
+  <si>
+    <t>Merit and availability of seats.</t>
+  </si>
+  <si>
+    <t>As notified.</t>
+  </si>
+  <si>
+    <t>Conducted only if officially notified by the University.</t>
+  </si>
+  <si>
+    <t>Student Services</t>
+  </si>
+  <si>
+    <t>Hostel Admission</t>
+  </si>
+  <si>
+    <t>Eligible Students</t>
+  </si>
+  <si>
+    <t>Hostel accommodation is available only in selected constituent colleges and is allotted subject to availability and institutional rules.</t>
+  </si>
+  <si>
+    <t>Hostel application form, admission proof, identity proof and other documents as prescribed.</t>
+  </si>
+  <si>
+    <t>Subject to admission in the college and hostel rules.</t>
+  </si>
+  <si>
+    <t>Offline / Online (College-specific)</t>
+  </si>
+  <si>
+    <t>Availability of hostel seats and college norms.</t>
+  </si>
+  <si>
+    <t>As per hostel policy, where applicable.</t>
+  </si>
+  <si>
+    <t>As notified by the concerned college.</t>
+  </si>
+  <si>
+    <t>Concerned Constituent College</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Hostel facilities are </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>not available in all constituent colleges</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Students should verify availability with the respective college.</t>
+    </r>
+  </si>
+  <si>
+    <t>Official College Websites</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -85,6 +478,27 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0D0D0D"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0D0D0D"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -111,16 +525,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -423,123 +856,747 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="46.28515625" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" customWidth="1"/>
+    <col min="5" max="5" width="19.140625" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" customWidth="1"/>
+    <col min="8" max="8" width="18.85546875" customWidth="1"/>
+    <col min="9" max="12" width="17.140625" customWidth="1"/>
+    <col min="13" max="13" width="12.140625" customWidth="1"/>
+    <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="15" max="15" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="N1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
+    </row>
+    <row r="2" spans="1:15" ht="179.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="169.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" t="s">
+      <c r="O3" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="N4" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>60</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" ht="75" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="5" spans="1:15" ht="121.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="N5" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="O5" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="120.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="4">
-        <v>46226</v>
+      <c r="B6" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="N6" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="90" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="7" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="N7" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="4">
-        <v>46226</v>
+      <c r="O7" s="8" t="s">
+        <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="8" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="N8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="4">
-        <v>46226</v>
+      <c r="O8" s="8" t="s">
+        <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="9" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="N9" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="4">
-        <v>46226</v>
+      <c r="O9" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="N10" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="O10" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="N11" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="O11" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="N12" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="O12" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="N13" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="O13" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="N14" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="O14" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="N15" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="O15" s="8" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E5" r:id="rId1"/>
-    <hyperlink ref="C5" r:id="rId2"/>
+    <hyperlink ref="M2" r:id="rId1" display="https://cuet.nta.nic.in"/>
+    <hyperlink ref="N2" r:id="rId2" display="https://cuet.nta.nic.in"/>
+    <hyperlink ref="N4" r:id="rId3"/>
+    <hyperlink ref="N5" r:id="rId4"/>
+    <hyperlink ref="N6" r:id="rId5"/>
+    <hyperlink ref="N7" r:id="rId6"/>
+    <hyperlink ref="N12" r:id="rId7"/>
+    <hyperlink ref="N8" r:id="rId8"/>
+    <hyperlink ref="N9" r:id="rId9"/>
+    <hyperlink ref="N10" r:id="rId10"/>
+    <hyperlink ref="N11" r:id="rId11"/>
+    <hyperlink ref="N13" r:id="rId12"/>
+    <hyperlink ref="N14" r:id="rId13"/>
+    <hyperlink ref="N15" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId15"/>
 </worksheet>
 </file>
 

</xml_diff>